<commit_message>
Fixes For Failed Test Scenarios Of Sales Order Screen
Fixes For Failed Test Scenarios Of Sales Order Screen
</commit_message>
<xml_diff>
--- a/testdata/QA Scenario - Sales STD PRICE.xlsx
+++ b/testdata/QA Scenario - Sales STD PRICE.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="16215" windowHeight="5535" firstSheet="5" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="16215" windowHeight="5535"/>
   </bookViews>
   <sheets>
     <sheet name="Case 1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="93">
   <si>
     <t>Item</t>
   </si>
@@ -1388,86 +1388,86 @@
       <c r="L5" s="33">
         <v>0</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>15000</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>15000</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>0</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>0</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>15000</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>1800</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>1800</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5" si="0">U5+AA5</f>
         <v>16800</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5" si="1">U5*$N$3</f>
         <v>15000</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
-      <c r="AG5" s="38" t="s">
+      <c r="AG5" t="s" s="38">
         <v>87</v>
       </c>
-      <c r="AH5" s="38" t="s">
+      <c r="AH5" t="s" s="38">
         <v>55</v>
       </c>
       <c r="AI5" s="29">
@@ -1526,91 +1526,91 @@
       <c r="L6" s="33">
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>20000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>20000</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>N6+P6+R6</f>
         <v>0</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>0</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>20000</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
         <v>1000</v>
       </c>
-      <c r="AA6" s="29">
+      <c r="AA6" s="33">
         <f>X6+Y6+Z6</f>
         <v>1000</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" ref="AB6" si="3">U6+AA6</f>
         <v>21000</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" ref="AD6" si="4">U6*$N$3</f>
         <v>20000</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
-      <c r="AG6" s="38" t="s">
+      <c r="AG6" t="s" s="38">
         <v>88</v>
       </c>
-      <c r="AH6" s="38" t="s">
+      <c r="AH6" t="s" s="38">
         <v>56</v>
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>1375.002</v>
+        <v>1371.6690000000001</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>50</v>
@@ -1723,7 +1723,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:AM8"/>
+  <dimension ref="A1:AM12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" style="1" width="5.7109375"/>
@@ -2046,57 +2046,57 @@
       <c r="L5" s="33">
         <v>10</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>1500</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>13500</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>1350</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>12150</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>1215</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>ROUND(N5+P5+R5,2)</f>
         <v>4065</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>406.5</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>10935</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>1312.2</v>
       </c>
@@ -2104,21 +2104,21 @@
         <f>ROUND((X5+Y5+Z5+AM5),2)</f>
         <v>1312.2</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
         <v>12247.2</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
         <v>10935</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f>G5/AE5</f>
         <v>10</v>
       </c>
@@ -2184,57 +2184,57 @@
       <c r="L6" s="33">
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>20000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>20000</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>ROUND(N6+P6+R6,2)</f>
         <v>0</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>0</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>20000</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.12</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
         <v>2400</v>
       </c>
@@ -2242,21 +2242,21 @@
         <f>ROUND((X6+Y6+Z6+AM6),2)</f>
         <v>3600</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" si="0"/>
         <v>23600</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -2367,6 +2367,9 @@
       <c r="AF8" s="13"/>
       <c r="AG8" s="13"/>
       <c r="AH8" s="13"/>
+    </row>
+    <row r="12" spans="1:39">
+      <c r="J12" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2707,39 +2710,39 @@
       <c r="L5" s="33">
         <v>0</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>15000</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>15000</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>0</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>0</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>15000</v>
       </c>
@@ -2749,37 +2752,37 @@
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>1800</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>1800</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
         <v>16800</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
         <v>15000</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -2846,39 +2849,39 @@
       <c r="L6" s="33">
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>20000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>20000</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>N6+P6+R6</f>
         <v>0</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>0</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>20000</v>
       </c>
@@ -2888,37 +2891,37 @@
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
         <v>1000</v>
       </c>
-      <c r="AA6" s="29">
+      <c r="AA6" s="33">
         <f>X6+Y6+Z6</f>
         <v>1000</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" si="0"/>
         <v>21000</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -2930,7 +2933,7 @@
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>1375.002</v>
+        <v>1371.6690000000001</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>50</v>
@@ -5218,79 +5221,79 @@
       <c r="L5" s="33">
         <v>0</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>15000</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>15000</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>0</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>0</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>15000</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>1800</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>1800</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
         <v>16800</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
         <v>15000</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -5356,79 +5359,79 @@
       <c r="L6" s="33">
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>20000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>20000</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>N6+P6+R6</f>
         <v>0</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>0</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>20000</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
         <v>1000</v>
       </c>
-      <c r="AA6" s="29">
+      <c r="AA6" s="33">
         <f>X6+Y6+Z6</f>
         <v>1000</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" si="0"/>
         <v>21000</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -5440,7 +5443,7 @@
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>1375.002</v>
+        <v>1371.6690000000001</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>50</v>
@@ -5876,79 +5879,79 @@
       <c r="L5" s="33">
         <v>0</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>15000</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>15000</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>0</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>0</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>15000</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>1800</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>1800</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
         <v>16800</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
         <v>15000</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -6014,79 +6017,79 @@
       <c r="L6" s="33">
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>20000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>20000</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>N6+P6+R6</f>
         <v>0</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>0</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>20000</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
         <v>1000</v>
       </c>
-      <c r="AA6" s="29">
+      <c r="AA6" s="33">
         <f>X6+Y6+Z6</f>
         <v>1000</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" si="0"/>
         <v>21000</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -6098,7 +6101,7 @@
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>1375.002</v>
+        <v>1371.6690000000001</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>50</v>
@@ -6534,79 +6537,79 @@
       <c r="L5" s="33">
         <v>20</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>1500</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>13500</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>2025</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>11475</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>2295</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>5820</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>582</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>9180</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.05</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>459</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>459</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5" si="0">U5+AA5</f>
         <v>9639</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5" si="1">U5*$N$3</f>
         <v>9180</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -7061,79 +7064,79 @@
       <c r="L5" s="33">
         <v>20</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>1500</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>13500</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>2025</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>11475</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>2295</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>5820</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>582</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>9180</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.05</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>459</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>459</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5" si="0">U5+AA5</f>
         <v>9639</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5" si="1">U5*$N$3</f>
         <v>9180</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -7588,79 +7591,79 @@
       <c r="L5" s="33">
         <v>20</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>1500</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>13500</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>1620</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>11880</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>2376</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>N5+P5+R5</f>
         <v>5496</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>549.6</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>9504</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>ROUND(IF($D$3=2,((U5*W5)),0),2)</f>
         <v>1140.48</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>1140.48</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
         <v>10644.48</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
         <v>9504</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -7726,79 +7729,79 @@
       <c r="L6" s="33">
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>20000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>20000</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>N6+P6+R6</f>
         <v>0</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>0</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>20000</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>0</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>ROUND(IF($D$3=2,((U6*W6)),0),2)</f>
         <v>1000</v>
       </c>
-      <c r="AA6" s="29">
+      <c r="AA6" s="33">
         <f>X6+Y6+Z6</f>
         <v>1000</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" si="0"/>
         <v>21000</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -7810,7 +7813,7 @@
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>1375.002</v>
+        <v>-3.3330000000000002</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>59</v>
@@ -8246,79 +8249,79 @@
       <c r="L5" s="33">
         <v>10</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>1500</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>13500</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>1350</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>12150</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>1215</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>ROUND(N5+P5+R5,2)</f>
         <v>4065</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>406.5</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>10935</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>656.1</v>
       </c>
-      <c r="Y5" s="29">
+      <c r="Y5" s="33">
         <f>IF($D$3=1,ROUND(((U5*W5)/2),2),0)</f>
         <v>656.1</v>
       </c>
-      <c r="Z5" s="29">
+      <c r="Z5" s="33">
         <f>IF($D$3=2,ROUND(((U5*W5)),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA5" s="29">
+      <c r="AA5" s="33">
         <f>X5+Y5+Z5</f>
         <v>1312.2</v>
       </c>
-      <c r="AB5" s="29">
+      <c r="AB5" s="33">
         <f t="shared" ref="AB5:AB6" si="0">U5+AA5</f>
         <v>12247.2</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="1">U5*$N$3</f>
         <v>10935</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="2">G5/AE5</f>
         <v>10</v>
       </c>
@@ -8384,79 +8387,79 @@
       <c r="L6" s="33">
         <v>10</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>2000</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>18000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>1800</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>16200</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>1620</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>ROUND(N6+P6+R6,2)</f>
         <v>5420</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>542</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>14580</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>364.5</v>
       </c>
-      <c r="Y6" s="29">
+      <c r="Y6" s="33">
         <f>IF($D$3=1,ROUND(((U6*W6)/2),2),0)</f>
         <v>364.5</v>
       </c>
-      <c r="Z6" s="29">
+      <c r="Z6" s="33">
         <f>IF($D$3=2,ROUND(((U6*W6)),2),0)</f>
         <v>0</v>
       </c>
-      <c r="AA6" s="29">
+      <c r="AA6" s="33">
         <f>X6+Y6+Z6</f>
         <v>729</v>
       </c>
-      <c r="AB6" s="29">
+      <c r="AB6" s="33">
         <f t="shared" si="0"/>
         <v>15309</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="1"/>
         <v>14580</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -8468,7 +8471,7 @@
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>-3.3330000000000002</v>
+        <v>1371.6690000000001</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>50</v>
@@ -8904,75 +8907,75 @@
       <c r="L5" s="33">
         <v>10</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="33">
         <f>I5</f>
         <v>15000</v>
       </c>
-      <c r="N5" s="29">
+      <c r="N5" s="33">
         <f>ROUND((M5*J5)/100,2)</f>
         <v>1500</v>
       </c>
-      <c r="O5" s="29">
+      <c r="O5" s="33">
         <f>I5-N5</f>
         <v>13500</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="33">
         <f>ROUND((O5*K5)/100,2)</f>
         <v>1350</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="33">
         <f>ROUND(O5-P5,2)</f>
         <v>12150</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="33">
         <f>ROUND((Q5*L5)/100,2)</f>
         <v>1215</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="33">
         <f>ROUND(N5+P5+R5,2)</f>
         <v>4065</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="33">
         <f>S5/G5</f>
         <v>406.5</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="33">
         <f>(I5-S5)</f>
         <v>10935</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W5" s="30">
         <v>0.12</v>
       </c>
-      <c r="X5" s="29">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="29">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="29">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="29">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="29">
+      <c r="X5" s="33">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="33">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="33">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="33">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="33">
         <f>U5+AA5</f>
         <v>10935</v>
       </c>
-      <c r="AC5" s="29">
+      <c r="AC5" s="33">
         <v>120</v>
       </c>
-      <c r="AD5" s="29">
+      <c r="AD5" s="33">
         <f t="shared" ref="AD5:AD6" si="0">U5*$N$3</f>
         <v>10935</v>
       </c>
-      <c r="AE5" s="32">
+      <c r="AE5" s="33">
         <v>1</v>
       </c>
-      <c r="AF5" s="29">
+      <c r="AF5" s="33">
         <f t="shared" ref="AF5" si="1">G5/AE5</f>
         <v>10</v>
       </c>
@@ -9038,75 +9041,75 @@
       <c r="L6" s="33">
         <v>10</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="33">
         <f>I6</f>
         <v>20000</v>
       </c>
-      <c r="N6" s="29">
+      <c r="N6" s="33">
         <f>ROUND((M6*J6)/100,2)</f>
         <v>2000</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6" s="33">
         <f>I6-N6</f>
         <v>18000</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="33">
         <f>ROUND((O6*K6)/100,2)</f>
         <v>1800</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="33">
         <f>ROUND(O6-P6,2)</f>
         <v>16200</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="33">
         <f>ROUND((Q6*L6)/100,2)</f>
         <v>1620</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="33">
         <f>ROUND(N6+P6+R6,2)</f>
         <v>5420</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="33">
         <f>S6/G6</f>
         <v>542</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="33">
         <f>(I6-S6)</f>
         <v>14580</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="33" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="30">
         <v>0.05</v>
       </c>
-      <c r="X6" s="29">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="29">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="29">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="29">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="29">
+      <c r="X6" s="33">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="33">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="33">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="33">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="33">
         <f t="shared" ref="AB6" si="2">U6+AA6</f>
         <v>14580</v>
       </c>
-      <c r="AC6" s="29">
+      <c r="AC6" s="33">
         <v>120</v>
       </c>
-      <c r="AD6" s="29">
+      <c r="AD6" s="33">
         <f t="shared" si="0"/>
         <v>14580</v>
       </c>
-      <c r="AE6" s="32">
+      <c r="AE6" s="33">
         <v>3</v>
       </c>
-      <c r="AF6" s="32">
+      <c r="AF6" s="33">
         <f>ROUND(G6/AE6,3)</f>
         <v>3.3330000000000002</v>
       </c>
@@ -9118,7 +9121,7 @@
       </c>
       <c r="AI6" s="29">
         <f>ROUND((AG6-AF6),3)</f>
-        <v>1375.002</v>
+        <v>1371.6690000000001</v>
       </c>
       <c r="AJ6" s="27" t="s">
         <v>50</v>

</xml_diff>

<commit_message>
Updated Sales Order Loators And Functions
Updated Sales Order Loators And Functions
</commit_message>
<xml_diff>
--- a/testdata/QA Scenario - Sales STD PRICE.xlsx
+++ b/testdata/QA Scenario - Sales STD PRICE.xlsx
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4351" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4381" uniqueCount="207">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -2229,7 +2229,9 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="J2" t="s" s="4">
+        <v>52</v>
+      </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -2271,8 +2273,8 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="9"/>
-      <c r="J3" s="10" t="s">
-        <v>4</v>
+      <c r="J3" t="s" s="4">
+        <v>62</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>5</v>
@@ -2458,7 +2460,7 @@
       <c r="G5" s="23">
         <v>44</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>51</v>
       </c>
       <c r="I5" s="23">
@@ -2610,7 +2612,7 @@
       <c r="G6" s="23">
         <v>53</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>61</v>
       </c>
       <c r="I6" s="23">
@@ -2932,7 +2934,9 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="J2" t="s" s="4">
+        <v>62</v>
+      </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -2974,8 +2978,8 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="9"/>
-      <c r="J3" s="10" t="s">
-        <v>4</v>
+      <c r="J3" t="s" s="4">
+        <v>95</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>5</v>
@@ -3161,7 +3165,7 @@
       <c r="G5" s="23">
         <v>10</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>93</v>
       </c>
       <c r="I5" s="23">
@@ -3313,7 +3317,7 @@
       <c r="G6" s="23">
         <v>10</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>94</v>
       </c>
       <c r="I6" s="23">
@@ -9024,7 +9028,9 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="J2" t="s" s="4">
+        <v>52</v>
+      </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -9066,8 +9072,8 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="9"/>
-      <c r="J3" s="10" t="s">
-        <v>4</v>
+      <c r="J3" t="s" s="4">
+        <v>62</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>5</v>
@@ -9253,7 +9259,7 @@
       <c r="G5" s="23">
         <v>5</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>68</v>
       </c>
       <c r="I5" s="23">
@@ -9404,7 +9410,7 @@
       <c r="G6" s="23">
         <v>89</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>69</v>
       </c>
       <c r="I6" s="23">
@@ -17217,7 +17223,7 @@
       <c r="G5" s="23">
         <v>21</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>71</v>
       </c>
       <c r="I5" s="23">
@@ -17369,7 +17375,7 @@
       <c r="G6" s="23">
         <v>35</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>73</v>
       </c>
       <c r="I6" s="23">
@@ -29674,7 +29680,7 @@
       <c r="G5" s="23">
         <v>11</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>74</v>
       </c>
       <c r="I5" s="23">
@@ -29825,7 +29831,7 @@
       <c r="G6" s="23">
         <v>15</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>75</v>
       </c>
       <c r="I6" s="23">
@@ -39576,7 +39582,7 @@
       <c r="G5" s="23">
         <v>22</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>77</v>
       </c>
       <c r="I5" s="23">
@@ -39727,7 +39733,7 @@
       <c r="G6" s="23">
         <v>12</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>79</v>
       </c>
       <c r="I6" s="23">
@@ -42961,7 +42967,7 @@
       <c r="G5" s="23">
         <v>12</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>80</v>
       </c>
       <c r="I5" s="23">
@@ -43113,7 +43119,7 @@
       <c r="G6" s="23">
         <v>14</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>81</v>
       </c>
       <c r="I6" s="23">
@@ -43435,7 +43441,9 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="J2" t="s" s="4">
+        <v>62</v>
+      </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -43477,8 +43485,8 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="9"/>
-      <c r="J3" s="10" t="s">
-        <v>4</v>
+      <c r="J3" t="s" s="4">
+        <v>52</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>5</v>
@@ -43664,7 +43672,7 @@
       <c r="G5" s="23">
         <v>10</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>69</v>
       </c>
       <c r="I5" s="23">
@@ -43815,7 +43823,7 @@
       <c r="G6" s="23">
         <v>10</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>74</v>
       </c>
       <c r="I6" s="23">

</xml_diff>

<commit_message>
Updated The Sales Order And Amendment Functions
Updated The Sales Order And Amendment Functions
</commit_message>
<xml_diff>
--- a/testdata/QA Scenario - Sales STD PRICE.xlsx
+++ b/testdata/QA Scenario - Sales STD PRICE.xlsx
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4146" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4174" uniqueCount="201">
   <si>
     <t>Scenario  : Local Sales - Stock UOM and Sales UOM (Similar)   DOC NO :  SORD-2425-00089</t>
   </si>
@@ -1871,14 +1871,14 @@
       <c r="G5" s="23">
         <v>44</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>51</v>
       </c>
       <c r="I5" s="23">
         <f>ROUND(G5*H5,2)</f>
         <v>73700</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" t="s" s="4">
         <v>52</v>
       </c>
       <c r="K5" s="23">
@@ -2023,14 +2023,14 @@
       <c r="G6" s="23">
         <v>53</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>61</v>
       </c>
       <c r="I6" s="23">
         <f>ROUND(G6*H6,2)</f>
         <v>171879</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" t="s" s="4">
         <v>62</v>
       </c>
       <c r="K6" s="23">
@@ -2568,14 +2568,14 @@
       <c r="G5" s="23">
         <v>10</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>91</v>
       </c>
       <c r="I5" s="23">
         <f>G5*H5</f>
         <v>21800</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" t="s" s="4">
         <v>62</v>
       </c>
       <c r="K5" s="23">
@@ -2720,14 +2720,14 @@
       <c r="G6" s="23">
         <v>10</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>92</v>
       </c>
       <c r="I6" s="23">
         <f>G6*H6</f>
         <v>31200</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" t="s" s="4">
         <v>93</v>
       </c>
       <c r="K6" s="23">
@@ -8644,14 +8644,14 @@
       <c r="G5" s="23">
         <v>5</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>68</v>
       </c>
       <c r="I5" s="23">
         <f>ROUND(G5*H5,2)</f>
         <v>120</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" t="s" s="4">
         <v>52</v>
       </c>
       <c r="K5" s="23">
@@ -8795,14 +8795,14 @@
       <c r="G6" s="23">
         <v>89</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>69</v>
       </c>
       <c r="I6" s="23">
         <f>ROUND(G6*H6,2)</f>
         <v>2670</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" t="s" s="4">
         <v>62</v>
       </c>
       <c r="K6" s="23">
@@ -16594,7 +16594,7 @@
       <c r="G5" s="23">
         <v>21</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>71</v>
       </c>
       <c r="I5" s="23">
@@ -16746,7 +16746,7 @@
       <c r="G6" s="23">
         <v>35</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>73</v>
       </c>
       <c r="I6" s="23">
@@ -29029,7 +29029,7 @@
       <c r="G5" s="23">
         <v>11</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>74</v>
       </c>
       <c r="I5" s="23">
@@ -29180,7 +29180,7 @@
       <c r="G6" s="23">
         <v>15</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>75</v>
       </c>
       <c r="I6" s="23">
@@ -38909,7 +38909,7 @@
       <c r="G5" s="23">
         <v>22</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>77</v>
       </c>
       <c r="I5" s="23">
@@ -39060,7 +39060,7 @@
       <c r="G6" s="23">
         <v>12</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>79</v>
       </c>
       <c r="I6" s="23">
@@ -42288,7 +42288,7 @@
       <c r="G5" s="23">
         <v>12</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>80</v>
       </c>
       <c r="I5" s="23">
@@ -42440,7 +42440,7 @@
       <c r="G6" s="23">
         <v>14</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>81</v>
       </c>
       <c r="I6" s="23">
@@ -42991,14 +42991,14 @@
       <c r="G5" s="23">
         <v>10</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" t="s" s="4">
         <v>69</v>
       </c>
       <c r="I5" s="23">
         <f>ROUND(G5*H5,2)</f>
         <v>300</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" t="s" s="4">
         <v>62</v>
       </c>
       <c r="K5" s="23">
@@ -43142,14 +43142,14 @@
       <c r="G6" s="23">
         <v>10</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s" s="4">
         <v>74</v>
       </c>
       <c r="I6" s="23">
         <f>ROUND(G6*H6,2)</f>
         <v>250</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" t="s" s="4">
         <v>52</v>
       </c>
       <c r="K6" s="23">

</xml_diff>